<commit_message>
Atualizando dados W27, script e actions
</commit_message>
<xml_diff>
--- a/Visao_Executiva_BSC_Master_v4.xlsx
+++ b/Visao_Executiva_BSC_Master_v4.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="134">
   <si>
     <t>BCS - JM</t>
   </si>
@@ -98,12 +98,108 @@
     <t>96.08%</t>
   </si>
   <si>
+    <t>Pickup Sucess (Ontime) FULL</t>
+  </si>
+  <si>
+    <t>92.8%</t>
+  </si>
+  <si>
+    <t>89.53%</t>
+  </si>
+  <si>
+    <t>88.75%</t>
+  </si>
+  <si>
+    <t>93.37%</t>
+  </si>
+  <si>
+    <t>94.77%</t>
+  </si>
+  <si>
+    <t>84.13%</t>
+  </si>
+  <si>
+    <t>91.61%</t>
+  </si>
+  <si>
+    <t>Atingido</t>
+  </si>
+  <si>
+    <t>% Real x D7 FDS (SVC) SPOT</t>
+  </si>
+  <si>
+    <t>90.0%</t>
+  </si>
+  <si>
+    <t>54.55%</t>
+  </si>
+  <si>
+    <t>66.67%</t>
+  </si>
+  <si>
+    <t>58.33%</t>
+  </si>
+  <si>
+    <t>75.00%</t>
+  </si>
+  <si>
+    <t>9.09%</t>
+  </si>
+  <si>
+    <t>63.64%</t>
+  </si>
+  <si>
+    <t>Aderência ao Perfil FULL</t>
+  </si>
+  <si>
+    <t>95.0%</t>
+  </si>
+  <si>
+    <t>98.47%</t>
+  </si>
+  <si>
+    <t>94.70%</t>
+  </si>
+  <si>
+    <t>97.87%</t>
+  </si>
+  <si>
+    <t>96.53%</t>
+  </si>
+  <si>
+    <t>99.36%</t>
+  </si>
+  <si>
+    <t>96.89%</t>
+  </si>
+  <si>
+    <t>Aceite Scheduling Pré Routing</t>
+  </si>
+  <si>
+    <t>5.0%</t>
+  </si>
+  <si>
+    <t>5.03%</t>
+  </si>
+  <si>
+    <t>3.78%</t>
+  </si>
+  <si>
+    <t>4.14%</t>
+  </si>
+  <si>
+    <t>3.95%</t>
+  </si>
+  <si>
+    <t>1.91%</t>
+  </si>
+  <si>
+    <t>4.23%</t>
+  </si>
+  <si>
     <t>% Utilização Frota Fixa FULL</t>
   </si>
   <si>
-    <t>95.0%</t>
-  </si>
-  <si>
     <t>89.46%</t>
   </si>
   <si>
@@ -122,28 +218,52 @@
     <t>86.26%</t>
   </si>
   <si>
-    <t>% Real x D7 FDS (SVC) SPOT</t>
-  </si>
-  <si>
-    <t>90.0%</t>
-  </si>
-  <si>
-    <t>54.55%</t>
-  </si>
-  <si>
-    <t>66.67%</t>
-  </si>
-  <si>
-    <t>58.33%</t>
-  </si>
-  <si>
-    <t>75.00%</t>
-  </si>
-  <si>
-    <t>9.09%</t>
-  </si>
-  <si>
-    <t>63.64%</t>
+    <t>SDD - % ER</t>
+  </si>
+  <si>
+    <t>91.83%</t>
+  </si>
+  <si>
+    <t>95.76%</t>
+  </si>
+  <si>
+    <t>89.78%</t>
+  </si>
+  <si>
+    <t>87.50%</t>
+  </si>
+  <si>
+    <t>0.00%</t>
+  </si>
+  <si>
+    <t>91.22%</t>
+  </si>
+  <si>
+    <t>Aceite de Scheduling XD</t>
+  </si>
+  <si>
+    <t>95.5%</t>
+  </si>
+  <si>
+    <t>86.76%</t>
+  </si>
+  <si>
+    <t>82.28%</t>
+  </si>
+  <si>
+    <t>98.00%</t>
+  </si>
+  <si>
+    <t>99.90%</t>
+  </si>
+  <si>
+    <t>76.62%</t>
+  </si>
+  <si>
+    <t>91.73%</t>
+  </si>
+  <si>
+    <t>% Utilização Frota Fixa (LM)</t>
   </si>
   <si>
     <t>Ad. Config XD</t>
@@ -155,39 +275,9 @@
     <t>107.85%</t>
   </si>
   <si>
-    <t>3012.14%</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
-    <t>1559.99%</t>
-  </si>
-  <si>
-    <t>SDD - % ER</t>
-  </si>
-  <si>
-    <t>91.83%</t>
-  </si>
-  <si>
-    <t>95.76%</t>
-  </si>
-  <si>
-    <t>89.78%</t>
-  </si>
-  <si>
-    <t>87.50%</t>
-  </si>
-  <si>
-    <t>0.00%</t>
-  </si>
-  <si>
-    <t>91.22%</t>
-  </si>
-  <si>
-    <t>% Utilização Frota Fixa (LM)</t>
-  </si>
-  <si>
     <t>Delivery Success XPT</t>
   </si>
   <si>
@@ -206,37 +296,37 @@
     <t>95.03%</t>
   </si>
   <si>
+    <t>% Real x D7 FDS (XPT) SPOT</t>
+  </si>
+  <si>
+    <t>100.00%</t>
+  </si>
+  <si>
+    <t>40.00%</t>
+  </si>
+  <si>
+    <t>60.00%</t>
+  </si>
+  <si>
+    <t>Telemetria MM XPT</t>
+  </si>
+  <si>
+    <t>72.0%</t>
+  </si>
+  <si>
+    <t>72.20%</t>
+  </si>
+  <si>
+    <t>54.00%</t>
+  </si>
+  <si>
+    <t>58.38%</t>
+  </si>
+  <si>
+    <t>61.53%</t>
+  </si>
+  <si>
     <t>Safety</t>
-  </si>
-  <si>
-    <t>% Real x D7 FDS (XPT) SPOT</t>
-  </si>
-  <si>
-    <t>100.00%</t>
-  </si>
-  <si>
-    <t>40.00%</t>
-  </si>
-  <si>
-    <t>60.00%</t>
-  </si>
-  <si>
-    <t>Telemetria MM XPT</t>
-  </si>
-  <si>
-    <t>72.0%</t>
-  </si>
-  <si>
-    <t>72.20%</t>
-  </si>
-  <si>
-    <t>54.00%</t>
-  </si>
-  <si>
-    <t>58.38%</t>
-  </si>
-  <si>
-    <t>61.53%</t>
   </si>
   <si>
     <t>Ad. Vec Fleet</t>
@@ -325,66 +415,6 @@
   </si>
   <si>
     <t>W26 (Fechamento)</t>
-  </si>
-  <si>
-    <t>Pickup Sucess (Ontime) FULL</t>
-  </si>
-  <si>
-    <t>92.8%</t>
-  </si>
-  <si>
-    <t>91.61%</t>
-  </si>
-  <si>
-    <t>94.77%</t>
-  </si>
-  <si>
-    <t>Atingido</t>
-  </si>
-  <si>
-    <t>84.13%</t>
-  </si>
-  <si>
-    <t>Aderência ao Perfil FULL</t>
-  </si>
-  <si>
-    <t>96.89%</t>
-  </si>
-  <si>
-    <t>96.53%</t>
-  </si>
-  <si>
-    <t>99.36%</t>
-  </si>
-  <si>
-    <t>Aceite de Scheduling XD</t>
-  </si>
-  <si>
-    <t>95.5%</t>
-  </si>
-  <si>
-    <t>91.73%</t>
-  </si>
-  <si>
-    <t>99.90%</t>
-  </si>
-  <si>
-    <t>76.62%</t>
-  </si>
-  <si>
-    <t>Aceite Scheduling Pré Routing</t>
-  </si>
-  <si>
-    <t>5.0%</t>
-  </si>
-  <si>
-    <t>4.23%</t>
-  </si>
-  <si>
-    <t>3.95%</t>
-  </si>
-  <si>
-    <t>1.91%</t>
   </si>
 </sst>
 </file>
@@ -1007,7 +1037,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S23"/>
+  <dimension ref="A1:S26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1212,10 +1242,10 @@
       <c r="D7" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="9" t="s">
         <v>33</v>
       </c>
       <c r="G7" s="8" t="s">
@@ -1224,32 +1254,32 @@
       <c r="H7" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="I7" s="8" t="s">
-        <v>20</v>
+      <c r="I7" s="9" t="s">
+        <v>36</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M7" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N7" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="O7" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P7" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q7" s="8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="R7" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="S7" s="8" t="s">
         <v>20</v>
@@ -1257,414 +1287,528 @@
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C8" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="I8" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="M8" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="N8" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="O8" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="P8" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q8" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="R8" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="S8" s="9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="D8" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="I8" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="K8" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="L8" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="M8" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="N8" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="O8" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="P8" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="Q8" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="R8" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="S8" s="8" t="s">
+      <c r="C9" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="I9" s="8" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="9" spans="11:19" x14ac:dyDescent="0.25">
       <c r="K9" s="6" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="M9" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="N9" s="8" t="s">
-        <v>31</v>
+        <v>69</v>
+      </c>
+      <c r="N9" s="9" t="s">
+        <v>70</v>
       </c>
       <c r="O9" s="8" t="s">
-        <v>32</v>
+        <v>71</v>
       </c>
       <c r="P9" s="8" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="Q9" s="8" t="s">
-        <v>34</v>
+        <v>73</v>
       </c>
       <c r="R9" s="7" t="s">
-        <v>35</v>
+        <v>74</v>
       </c>
       <c r="S9" s="8" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="11:19" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="I10" s="9" t="s">
+        <v>36</v>
+      </c>
       <c r="K10" s="6" t="s">
-        <v>58</v>
+        <v>83</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="M10" s="8" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="N10" s="8" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="O10" s="8" t="s">
-        <v>26</v>
+        <v>64</v>
       </c>
       <c r="P10" s="8" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="Q10" s="8" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="R10" s="7" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="S10" s="8" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A11" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11"/>
+      <c r="A11" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I11" s="10" t="s">
+        <v>87</v>
+      </c>
       <c r="K11" s="6" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="M11" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="N11" s="9" t="s">
-        <v>66</v>
+        <v>22</v>
+      </c>
+      <c r="M11" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="N11" s="8" t="s">
+        <v>90</v>
       </c>
       <c r="O11" s="8" t="s">
-        <v>55</v>
+        <v>26</v>
       </c>
       <c r="P11" s="8" t="s">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="Q11" s="8" t="s">
-        <v>55</v>
+        <v>92</v>
       </c>
       <c r="R11" s="7" t="s">
-        <v>68</v>
+        <v>93</v>
       </c>
       <c r="S11" s="8" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="E12" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="G12" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H12" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="I12" s="12" t="s">
-        <v>11</v>
-      </c>
+    <row r="12" spans="11:19" x14ac:dyDescent="0.25">
       <c r="K12" s="6" t="s">
-        <v>69</v>
+        <v>94</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>70</v>
+        <v>38</v>
       </c>
       <c r="M12" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="N12" s="8" t="s">
-        <v>72</v>
+        <v>95</v>
+      </c>
+      <c r="N12" s="9" t="s">
+        <v>95</v>
       </c>
       <c r="O12" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="P12" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q12" s="7" t="s">
-        <v>48</v>
+      <c r="P12" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="Q12" s="8" t="s">
+        <v>73</v>
       </c>
       <c r="R12" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="S12" s="10" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="I13" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="S12" s="8" t="s">
         <v>20</v>
       </c>
     </row>
+    <row r="13" spans="11:19" x14ac:dyDescent="0.25">
+      <c r="K13" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="M13" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="N13" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="O13" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="P13" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q13" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="R13" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="S13" s="10" t="s">
+        <v>87</v>
+      </c>
+    </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="H14" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="I14" s="10" t="s">
-        <v>48</v>
-      </c>
+      <c r="A14" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="C15" s="8" t="s">
+      <c r="A15" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="G15" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="H15" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="I15" s="12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="I16" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="I17" s="10" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C18" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="F15" s="8" t="s">
+      <c r="D18" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="I18" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="13"/>
+      <c r="H22" s="13"/>
+      <c r="I22" s="13"/>
+      <c r="J22" s="13"/>
+      <c r="K22" s="13"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="D23" s="14"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="G23" s="14"/>
+      <c r="H23" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="I23" s="14"/>
+      <c r="J23" s="14"/>
+      <c r="K23" s="14" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B24" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="G15" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="I15" s="8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="13"/>
-      <c r="H19" s="13"/>
-      <c r="I19" s="13"/>
-      <c r="J19" s="13"/>
-      <c r="K19" s="13"/>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="B20" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="I20" s="14"/>
-      <c r="J20" s="14"/>
-      <c r="K20" s="14" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="7" t="s">
+      <c r="C24" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="G24" s="7"/>
+      <c r="H24" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="I24" s="7"/>
+      <c r="J24" s="7"/>
+      <c r="K24" s="7" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B21" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="G21" s="7"/>
-      <c r="H21" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="I21" s="7"/>
-      <c r="J21" s="7"/>
-      <c r="K21" s="7" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="G22" s="7"/>
-      <c r="H22" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="I22" s="7"/>
-      <c r="J22" s="7"/>
-      <c r="K22" s="7" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="C23" s="6" t="s">
+      <c r="B25" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="G23" s="7"/>
-      <c r="H23" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="I23" s="7"/>
-      <c r="J23" s="7"/>
-      <c r="K23" s="8" t="s">
-        <v>100</v>
+      <c r="C25" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="G25" s="7"/>
+      <c r="H25" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="I25" s="7"/>
+      <c r="J25" s="7"/>
+      <c r="K25" s="7" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="G26" s="7"/>
+      <c r="H26" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="I26" s="7"/>
+      <c r="J26" s="7"/>
+      <c r="K26" s="8" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -1672,20 +1816,20 @@
     <mergeCell ref="A1:S2"/>
     <mergeCell ref="A4:I4"/>
     <mergeCell ref="K4:S4"/>
-    <mergeCell ref="A11:I11"/>
-    <mergeCell ref="A19:K19"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="H20:J20"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="H21:J21"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="H22:J22"/>
+    <mergeCell ref="A14:I14"/>
+    <mergeCell ref="A22:K22"/>
     <mergeCell ref="C23:E23"/>
     <mergeCell ref="F23:G23"/>
     <mergeCell ref="H23:J23"/>
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="H24:J24"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="H25:J25"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="H26:J26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1707,7 +1851,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -1727,7 +1871,7 @@
     </row>
     <row r="4" ht="25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
-        <v>102</v>
+        <v>132</v>
       </c>
       <c r="B4" s="16" t="s">
         <v>3</v>
@@ -1739,7 +1883,7 @@
         <v>10</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>103</v>
+        <v>133</v>
       </c>
       <c r="F4" s="16" t="s">
         <v>11</v>
@@ -1776,22 +1920,22 @@
         <v>1</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>104</v>
+        <v>28</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>105</v>
+        <v>29</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>106</v>
+        <v>35</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>107</v>
+        <v>33</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>108</v>
+        <v>36</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>109</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1799,22 +1943,22 @@
         <v>1</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>110</v>
+        <v>45</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>111</v>
+        <v>52</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>112</v>
+        <v>50</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>108</v>
+        <v>36</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>113</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1822,22 +1966,22 @@
         <v>1</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>28</v>
+        <v>61</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>35</v>
+        <v>67</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>33</v>
+        <v>65</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>20</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>34</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1845,22 +1989,22 @@
         <v>1</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>114</v>
+        <v>75</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>115</v>
+        <v>76</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>117</v>
+        <v>80</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>108</v>
+        <v>36</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>118</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1868,22 +2012,22 @@
         <v>1</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>44</v>
+        <v>84</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>48</v>
+        <v>87</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>48</v>
+        <v>87</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>48</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1914,22 +2058,22 @@
         <v>2</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F12" s="8" t="s">
         <v>20</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1937,22 +2081,22 @@
         <v>2</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>119</v>
+        <v>53</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>120</v>
+        <v>54</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>121</v>
+        <v>60</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>122</v>
+        <v>58</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>20</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>123</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1960,22 +2104,22 @@
         <v>2</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>20</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1983,22 +2127,22 @@
         <v>2</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>57</v>
+        <v>83</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>35</v>
+        <v>67</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>33</v>
+        <v>65</v>
       </c>
       <c r="F15" s="8" t="s">
         <v>20</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>34</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -2006,22 +2150,22 @@
         <v>2</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>58</v>
+        <v>88</v>
       </c>
       <c r="C16" s="18" t="s">
         <v>22</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>63</v>
+        <v>93</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>61</v>
+        <v>91</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>20</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>62</v>
+        <v>92</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -2029,22 +2173,22 @@
         <v>2</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>65</v>
+        <v>94</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>68</v>
+        <v>97</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>67</v>
+        <v>96</v>
       </c>
       <c r="F17" s="8" t="s">
         <v>20</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -2052,91 +2196,91 @@
         <v>2</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>48</v>
+        <v>87</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>48</v>
+        <v>87</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>48</v>
+        <v>87</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>64</v>
+        <v>104</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>76</v>
+        <v>106</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>76</v>
+        <v>106</v>
       </c>
       <c r="F19" s="8" t="s">
         <v>20</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>76</v>
+        <v>106</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>64</v>
+        <v>104</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>77</v>
+        <v>107</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>78</v>
+        <v>108</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>48</v>
+        <v>87</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>48</v>
+        <v>87</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>48</v>
+        <v>87</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>64</v>
+        <v>104</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>79</v>
+        <v>109</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>80</v>
+        <v>110</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>85</v>
+        <v>115</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>83</v>
+        <v>113</v>
       </c>
       <c r="F21" s="8" t="s">
         <v>20</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>84</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adjust columns to show June and weeks W26-W29
</commit_message>
<xml_diff>
--- a/Visao_Executiva_BSC_Master_v4.xlsx
+++ b/Visao_Executiva_BSC_Master_v4.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="137">
   <si>
     <t>BCS - JM</t>
   </si>
@@ -29,7 +29,7 @@
     <t>Objetivo</t>
   </si>
   <si>
-    <t>W25</t>
+    <t>Junho</t>
   </si>
   <si>
     <t>W26</t>
@@ -56,7 +56,7 @@
     <t>97.9%</t>
   </si>
   <si>
-    <t>97.30%</t>
+    <t>96.85%</t>
   </si>
   <si>
     <t>97.69%</t>
@@ -71,7 +71,7 @@
     <t>88.67%</t>
   </si>
   <si>
-    <t>97.55%</t>
+    <t>97.44%</t>
   </si>
   <si>
     <t>Abaixo</t>
@@ -83,7 +83,7 @@
     <t>98.2%</t>
   </si>
   <si>
-    <t>96.07%</t>
+    <t>96.04%</t>
   </si>
   <si>
     <t>95.75%</t>
@@ -98,7 +98,7 @@
     <t>95.78%</t>
   </si>
   <si>
-    <t>96.11%</t>
+    <t>96.10%</t>
   </si>
   <si>
     <t>Pickup Sucess (Ontime) FULL</t>
@@ -107,7 +107,7 @@
     <t>92.6%</t>
   </si>
   <si>
-    <t>93.37%</t>
+    <t>91.75%</t>
   </si>
   <si>
     <t>94.82%</t>
@@ -122,7 +122,7 @@
     <t>86.06%</t>
   </si>
   <si>
-    <t>94.12%</t>
+    <t>93.72%</t>
   </si>
   <si>
     <t>Atingido</t>
@@ -134,7 +134,7 @@
     <t>90.0%</t>
   </si>
   <si>
-    <t>58.33%</t>
+    <t>69.23%</t>
   </si>
   <si>
     <t>75.00%</t>
@@ -149,7 +149,7 @@
     <t>0.00%</t>
   </si>
   <si>
-    <t>56.06%</t>
+    <t>58.78%</t>
   </si>
   <si>
     <t>% Utilização Frota Fixa FULL</t>
@@ -158,25 +158,28 @@
     <t>95.0%</t>
   </si>
   <si>
+    <t>86.68%</t>
+  </si>
+  <si>
+    <t>85.83%</t>
+  </si>
+  <si>
+    <t>82.54%</t>
+  </si>
+  <si>
     <t>84.96%</t>
   </si>
   <si>
-    <t>85.83%</t>
-  </si>
-  <si>
-    <t>82.54%</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
-    <t>84.57%</t>
+    <t>85.00%</t>
   </si>
   <si>
     <t>SDD - % ER</t>
   </si>
   <si>
-    <t>89.78%</t>
+    <t>90.46%</t>
   </si>
   <si>
     <t>86.82%</t>
@@ -191,13 +194,13 @@
     <t>56.78%</t>
   </si>
   <si>
-    <t>88.78%</t>
+    <t>88.95%</t>
   </si>
   <si>
     <t>Aceite de Scheduling XD</t>
   </si>
   <si>
-    <t>98.00%</t>
+    <t>92.70%</t>
   </si>
   <si>
     <t>99.90%</t>
@@ -212,7 +215,7 @@
     <t>64.78%</t>
   </si>
   <si>
-    <t>96.66%</t>
+    <t>95.33%</t>
   </si>
   <si>
     <t>% Utilização Frota Fixa (LM)</t>
@@ -227,6 +230,9 @@
     <t>97.0%</t>
   </si>
   <si>
+    <t>96.22%</t>
+  </si>
+  <si>
     <t>84.69%</t>
   </si>
   <si>
@@ -239,13 +245,13 @@
     <t>40.47%</t>
   </si>
   <si>
-    <t>94.64%</t>
+    <t>95.03%</t>
   </si>
   <si>
     <t>Delivery Success XPT</t>
   </si>
   <si>
-    <t>94.75%</t>
+    <t>94.99%</t>
   </si>
   <si>
     <t>95.01%</t>
@@ -260,16 +266,19 @@
     <t>89.00%</t>
   </si>
   <si>
-    <t>94.61%</t>
+    <t>94.67%</t>
   </si>
   <si>
     <t>% Real x D7 FDS (XPT) SPOT</t>
   </si>
   <si>
+    <t>80.00%</t>
+  </si>
+  <si>
     <t>40.00%</t>
   </si>
   <si>
-    <t>80.00%</t>
+    <t>60.00%</t>
   </si>
   <si>
     <t>Telemetria MM XPT</t>
@@ -278,7 +287,7 @@
     <t>72.0%</t>
   </si>
   <si>
-    <t>58.38%</t>
+    <t>64.50%</t>
   </si>
   <si>
     <t>63.55%</t>
@@ -290,7 +299,7 @@
     <t>67.91%</t>
   </si>
   <si>
-    <t>64.55%</t>
+    <t>66.08%</t>
   </si>
   <si>
     <t>Safety</t>
@@ -305,22 +314,19 @@
     <t>Telemetria Scorecard</t>
   </si>
   <si>
-    <t>88.17%</t>
-  </si>
-  <si>
     <t>81.32%</t>
   </si>
   <si>
     <t>87.47%</t>
   </si>
   <si>
-    <t>85.65%</t>
+    <t>84.58%</t>
   </si>
   <si>
     <t>Aderência Treinamentos Safety Driver</t>
   </si>
   <si>
-    <t>95.17%</t>
+    <t>96.41%</t>
   </si>
   <si>
     <t>96.23%</t>
@@ -333,6 +339,9 @@
   </si>
   <si>
     <t>96.68%</t>
+  </si>
+  <si>
+    <t>96.42%</t>
   </si>
   <si>
     <t>Acompanhamento de Ações / Status das Tarefas</t>
@@ -393,7 +402,7 @@
     <t>Aderência ao Perfil FULL</t>
   </si>
   <si>
-    <t>95.99%</t>
+    <t>95.73%</t>
   </si>
   <si>
     <t>93.13%</t>
@@ -408,7 +417,7 @@
     <t>5.0%</t>
   </si>
   <si>
-    <t>3.52%</t>
+    <t>3.48%</t>
   </si>
   <si>
     <t>4.39%</t>
@@ -1236,7 +1245,7 @@
       <c r="B7" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="8" t="s">
         <v>31</v>
       </c>
       <c r="D7" s="9" t="s">
@@ -1302,40 +1311,40 @@
         <v>50</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I8" s="8" t="s">
         <v>20</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L8" s="7" t="s">
         <v>47</v>
       </c>
       <c r="M8" s="8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="N8" s="8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="O8" s="8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="P8" s="8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q8" s="8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="R8" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="S8" s="8" t="s">
         <v>20</v>
@@ -1343,34 +1352,34 @@
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C9" s="9" t="s">
-        <v>61</v>
+      <c r="C9" s="8" t="s">
+        <v>62</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I9" s="8" t="s">
         <v>20</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="L9" s="7" t="s">
         <v>47</v>
@@ -1385,13 +1394,13 @@
         <v>50</v>
       </c>
       <c r="P9" s="8" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="Q9" s="8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="R9" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="S9" s="8" t="s">
         <v>20</v>
@@ -1399,55 +1408,55 @@
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>51</v>
+        <v>71</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>72</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="I10" s="9" t="s">
         <v>37</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="L10" s="7" t="s">
         <v>22</v>
       </c>
       <c r="M10" s="8" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="N10" s="8" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O10" s="8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="P10" s="8" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="Q10" s="8" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="R10" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="S10" s="8" t="s">
         <v>20</v>
@@ -1455,28 +1464,28 @@
     </row>
     <row r="11" spans="11:19" x14ac:dyDescent="0.25">
       <c r="K11" s="6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L11" s="7" t="s">
         <v>39</v>
       </c>
       <c r="M11" s="8" t="s">
-        <v>44</v>
+        <v>86</v>
       </c>
       <c r="N11" s="8" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="O11" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="P11" s="8" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="Q11" s="8" t="s">
         <v>44</v>
       </c>
       <c r="R11" s="7" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="S11" s="8" t="s">
         <v>20</v>
@@ -1484,28 +1493,28 @@
     </row>
     <row r="12" spans="11:19" x14ac:dyDescent="0.25">
       <c r="K12" s="6" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="M12" s="8" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="N12" s="8" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="O12" s="8" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="P12" s="8" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="Q12" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="R12" s="7" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="S12" s="8" t="s">
         <v>20</v>
@@ -1513,7 +1522,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -1555,86 +1564,86 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>39</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="I15" s="12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>39</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>97</v>
+        <v>51</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="I16" s="12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>28</v>
+        <v>109</v>
       </c>
       <c r="I17" s="8" t="s">
         <v>20</v>
@@ -1642,7 +1651,7 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
@@ -1657,22 +1666,22 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D22" s="14"/>
       <c r="E22" s="14"/>
       <c r="F22" s="14" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="G22" s="14"/>
       <c r="H22" s="14" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="I22" s="14"/>
       <c r="J22" s="14"/>
@@ -1685,24 +1694,24 @@
         <v>2</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
       <c r="F23" s="7" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="G23" s="7"/>
       <c r="H23" s="7" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="I23" s="7"/>
       <c r="J23" s="7"/>
       <c r="K23" s="7" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -1710,49 +1719,49 @@
         <v>2</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D24" s="6"/>
       <c r="E24" s="6"/>
       <c r="F24" s="7" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="G24" s="7"/>
       <c r="H24" s="7" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="I24" s="7"/>
       <c r="J24" s="7"/>
       <c r="K24" s="7" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D25" s="6"/>
       <c r="E25" s="6"/>
       <c r="F25" s="7" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="G25" s="7"/>
       <c r="H25" s="7" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="I25" s="7"/>
       <c r="J25" s="7"/>
       <c r="K25" s="8" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -1795,7 +1804,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -1815,7 +1824,7 @@
     </row>
     <row r="4" ht="25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B4" s="16" t="s">
         <v>3</v>
@@ -1827,7 +1836,7 @@
         <v>10</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F4" s="16" t="s">
         <v>11</v>
@@ -1887,22 +1896,22 @@
         <v>1</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C7" s="18" t="s">
         <v>47</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="F7" s="8" t="s">
         <v>20</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1916,16 +1925,16 @@
         <v>47</v>
       </c>
       <c r="D8" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="7" t="s">
         <v>52</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1933,22 +1942,22 @@
         <v>1</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C9" s="18" t="s">
         <v>47</v>
       </c>
       <c r="D9" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="G9" s="7" t="s">
         <v>66</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1956,22 +1965,22 @@
         <v>1</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D10" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="E10" s="9" t="s">
         <v>75</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>73</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>37</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -2025,22 +2034,22 @@
         <v>2</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>20</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -2048,22 +2057,22 @@
         <v>2</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C14" s="18" t="s">
         <v>47</v>
       </c>
       <c r="D14" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="G14" s="7" t="s">
         <v>59</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -2071,22 +2080,22 @@
         <v>2</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C15" s="18" t="s">
         <v>47</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F15" s="8" t="s">
         <v>20</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -2094,22 +2103,22 @@
         <v>2</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C16" s="18" t="s">
         <v>22</v>
       </c>
       <c r="D16" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="E16" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="E16" s="8" t="s">
-        <v>80</v>
-      </c>
       <c r="F16" s="8" t="s">
         <v>20</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -2117,16 +2126,16 @@
         <v>2</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C17" s="18" t="s">
         <v>39</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F17" s="8" t="s">
         <v>20</v>
@@ -2140,91 +2149,91 @@
         <v>2</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="F18" s="8" t="s">
         <v>20</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C19" s="18" t="s">
         <v>39</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C20" s="18" t="s">
         <v>39</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>28</v>
+        <v>109</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F21" s="8" t="s">
         <v>20</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao dos indicadores, correcao de nomes e remocao de duplicidades no BSC
</commit_message>
<xml_diff>
--- a/Visao_Executiva_BSC_Master_v4.xlsx
+++ b/Visao_Executiva_BSC_Master_v4.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="156">
   <si>
     <t>BCS - JM</t>
   </si>
@@ -29,22 +29,22 @@
     <t>Objetivo</t>
   </si>
   <si>
-    <t>W24</t>
-  </si>
-  <si>
-    <t>W25</t>
-  </si>
-  <si>
-    <t>W26</t>
-  </si>
-  <si>
-    <t>W27</t>
-  </si>
-  <si>
-    <t>W28</t>
-  </si>
-  <si>
-    <t>W29 (Prévia)</t>
+    <t>Fev</t>
+  </si>
+  <si>
+    <t>Mar</t>
+  </si>
+  <si>
+    <t>Abr</t>
+  </si>
+  <si>
+    <t>Mai</t>
+  </si>
+  <si>
+    <t>Junho</t>
+  </si>
+  <si>
+    <t>Jul</t>
   </si>
   <si>
     <t>Média</t>
@@ -56,28 +56,25 @@
     <t>Pickup Sucess (SI) FULL</t>
   </si>
   <si>
-    <t>97.9%</t>
-  </si>
-  <si>
-    <t>96.40%</t>
-  </si>
-  <si>
-    <t>97.30%</t>
-  </si>
-  <si>
-    <t>97.69%</t>
-  </si>
-  <si>
-    <t>97.86%</t>
-  </si>
-  <si>
-    <t>97.35%</t>
-  </si>
-  <si>
-    <t>88.67%</t>
-  </si>
-  <si>
-    <t>97.32%</t>
+    <t>97.4%</t>
+  </si>
+  <si>
+    <t>97.78%</t>
+  </si>
+  <si>
+    <t>98.39%</t>
+  </si>
+  <si>
+    <t>96.75%</t>
+  </si>
+  <si>
+    <t>96.85%</t>
+  </si>
+  <si>
+    <t>96.23%</t>
+  </si>
+  <si>
+    <t>97.51%</t>
   </si>
   <si>
     <t>Abaixo</t>
@@ -89,52 +86,52 @@
     <t>98.2%</t>
   </si>
   <si>
-    <t>96.07%</t>
-  </si>
-  <si>
-    <t>95.75%</t>
-  </si>
-  <si>
-    <t>96.24%</t>
-  </si>
-  <si>
-    <t>96.37%</t>
-  </si>
-  <si>
-    <t>95.78%</t>
-  </si>
-  <si>
-    <t>96.17%</t>
+    <t>95.96%</t>
+  </si>
+  <si>
+    <t>96.84%</t>
+  </si>
+  <si>
+    <t>96.56%</t>
+  </si>
+  <si>
+    <t>96.08%</t>
+  </si>
+  <si>
+    <t>96.04%</t>
+  </si>
+  <si>
+    <t>96.67%</t>
+  </si>
+  <si>
+    <t>96.30%</t>
   </si>
   <si>
     <t>Pickup Sucess (Ontime) FULL</t>
   </si>
   <si>
-    <t>92.6%</t>
-  </si>
-  <si>
-    <t>88.75%</t>
-  </si>
-  <si>
-    <t>93.37%</t>
-  </si>
-  <si>
-    <t>94.82%</t>
-  </si>
-  <si>
-    <t>94.29%</t>
-  </si>
-  <si>
-    <t>94.01%</t>
-  </si>
-  <si>
-    <t>86.06%</t>
-  </si>
-  <si>
-    <t>93.05%</t>
-  </si>
-  <si>
-    <t>Atingido</t>
+    <t>94.0%</t>
+  </si>
+  <si>
+    <t>95.63%</t>
+  </si>
+  <si>
+    <t>95.81%</t>
+  </si>
+  <si>
+    <t>97.11%</t>
+  </si>
+  <si>
+    <t>92.12%</t>
+  </si>
+  <si>
+    <t>91.75%</t>
+  </si>
+  <si>
+    <t>91.63%</t>
+  </si>
+  <si>
+    <t>94.48%</t>
   </si>
   <si>
     <t>% Real x D7 FDS (SVC) SPOT</t>
@@ -143,235 +140,265 @@
     <t>90.0%</t>
   </si>
   <si>
-    <t>66.67%</t>
-  </si>
-  <si>
     <t>58.33%</t>
   </si>
   <si>
+    <t>69.23%</t>
+  </si>
+  <si>
+    <t>53.85%</t>
+  </si>
+  <si>
+    <t>64.29%</t>
+  </si>
+  <si>
+    <t>18.18%</t>
+  </si>
+  <si>
+    <t>62.99%</t>
+  </si>
+  <si>
+    <t>% Utilização Frota Fixa FULL</t>
+  </si>
+  <si>
+    <t>95.0%</t>
+  </si>
+  <si>
+    <t>90.93%</t>
+  </si>
+  <si>
+    <t>90.55%</t>
+  </si>
+  <si>
+    <t>84.77%</t>
+  </si>
+  <si>
+    <t>83.69%</t>
+  </si>
+  <si>
+    <t>86.68%</t>
+  </si>
+  <si>
+    <t>79.31%</t>
+  </si>
+  <si>
+    <t>87.32%</t>
+  </si>
+  <si>
+    <t>SDD - % ER</t>
+  </si>
+  <si>
+    <t>80.60%</t>
+  </si>
+  <si>
+    <t>76.10%</t>
+  </si>
+  <si>
+    <t>68.25%</t>
+  </si>
+  <si>
+    <t>73.61%</t>
+  </si>
+  <si>
+    <t>90.46%</t>
+  </si>
+  <si>
+    <t>74.67%</t>
+  </si>
+  <si>
+    <t>77.80%</t>
+  </si>
+  <si>
+    <t>Aceite de Scheduling XD</t>
+  </si>
+  <si>
+    <t>99.25%</t>
+  </si>
+  <si>
+    <t>97.59%</t>
+  </si>
+  <si>
+    <t>99.21%</t>
+  </si>
+  <si>
+    <t>93.44%</t>
+  </si>
+  <si>
+    <t>92.70%</t>
+  </si>
+  <si>
+    <t>92.16%</t>
+  </si>
+  <si>
+    <t>96.44%</t>
+  </si>
+  <si>
+    <t>% Utilização Frota Fixa (LM)</t>
+  </si>
+  <si>
+    <t>Ad. Config XD</t>
+  </si>
+  <si>
+    <t>97.0%</t>
+  </si>
+  <si>
+    <t>104.55%</t>
+  </si>
+  <si>
+    <t>101.62%</t>
+  </si>
+  <si>
+    <t>103.26%</t>
+  </si>
+  <si>
+    <t>96.47%</t>
+  </si>
+  <si>
+    <t>96.22%</t>
+  </si>
+  <si>
+    <t>86.86%</t>
+  </si>
+  <si>
+    <t>100.42%</t>
+  </si>
+  <si>
+    <t>Delivery Success XPT</t>
+  </si>
+  <si>
+    <t>96.58%</t>
+  </si>
+  <si>
+    <t>95.97%</t>
+  </si>
+  <si>
+    <t>95.21%</t>
+  </si>
+  <si>
+    <t>94.99%</t>
+  </si>
+  <si>
+    <t>94.37%</t>
+  </si>
+  <si>
+    <t>95.71%</t>
+  </si>
+  <si>
+    <t>% Real x D7 FDS (XPT) SPOT</t>
+  </si>
+  <si>
+    <t>83.33%</t>
+  </si>
+  <si>
     <t>75.00%</t>
   </si>
   <si>
-    <t>54.55%</t>
-  </si>
-  <si>
-    <t>36.36%</t>
-  </si>
-  <si>
-    <t>0.00%</t>
-  </si>
-  <si>
-    <t>58.18%</t>
-  </si>
-  <si>
-    <t>% Utilização Frota Fixa FULL</t>
-  </si>
-  <si>
-    <t>95.0%</t>
-  </si>
-  <si>
-    <t>84.79%</t>
+    <t>80.00%</t>
+  </si>
+  <si>
+    <t>40.00%</t>
+  </si>
+  <si>
+    <t>80.33%</t>
+  </si>
+  <si>
+    <t>Telemetria MM XPT</t>
+  </si>
+  <si>
+    <t>72.0%</t>
+  </si>
+  <si>
+    <t>56.85%</t>
+  </si>
+  <si>
+    <t>120.44%</t>
+  </si>
+  <si>
+    <t>62.61%</t>
+  </si>
+  <si>
+    <t>67.31%</t>
+  </si>
+  <si>
+    <t>64.50%</t>
+  </si>
+  <si>
+    <t>50.49%</t>
+  </si>
+  <si>
+    <t>74.34%</t>
+  </si>
+  <si>
+    <t>Safety</t>
+  </si>
+  <si>
+    <t>Ad. Vec Fleet</t>
+  </si>
+  <si>
+    <t>83.68%</t>
+  </si>
+  <si>
+    <t>89.17%</t>
+  </si>
+  <si>
+    <t>51.68%</t>
+  </si>
+  <si>
+    <t>84.00%</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>78.51%</t>
+  </si>
+  <si>
+    <t>Telemetria Scorecard</t>
+  </si>
+  <si>
+    <t>85.0%</t>
+  </si>
+  <si>
+    <t>87.13%</t>
+  </si>
+  <si>
+    <t>169.17%</t>
+  </si>
+  <si>
+    <t>90.86%</t>
+  </si>
+  <si>
+    <t>78.40%</t>
   </si>
   <si>
     <t>84.96%</t>
   </si>
   <si>
-    <t>85.83%</t>
-  </si>
-  <si>
-    <t>82.54%</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>84.62%</t>
-  </si>
-  <si>
-    <t>SDD - % ER</t>
-  </si>
-  <si>
-    <t>95.76%</t>
-  </si>
-  <si>
-    <t>89.78%</t>
-  </si>
-  <si>
-    <t>86.82%</t>
-  </si>
-  <si>
-    <t>87.83%</t>
-  </si>
-  <si>
-    <t>90.71%</t>
-  </si>
-  <si>
-    <t>56.78%</t>
-  </si>
-  <si>
-    <t>90.18%</t>
-  </si>
-  <si>
-    <t>Aceite de Scheduling XD</t>
-  </si>
-  <si>
-    <t>82.28%</t>
-  </si>
-  <si>
-    <t>98.00%</t>
-  </si>
-  <si>
-    <t>99.90%</t>
-  </si>
-  <si>
-    <t>96.64%</t>
-  </si>
-  <si>
-    <t>92.08%</t>
-  </si>
-  <si>
-    <t>64.78%</t>
-  </si>
-  <si>
-    <t>93.78%</t>
-  </si>
-  <si>
-    <t>% Utilização Frota Fixa (LM)</t>
-  </si>
-  <si>
-    <t>44.41%</t>
-  </si>
-  <si>
-    <t>Ad. Config XD</t>
-  </si>
-  <si>
-    <t>97.0%</t>
-  </si>
-  <si>
-    <t>84.69%</t>
-  </si>
-  <si>
-    <t>99.60%</t>
-  </si>
-  <si>
-    <t>99.62%</t>
-  </si>
-  <si>
-    <t>40.47%</t>
-  </si>
-  <si>
-    <t>94.64%</t>
-  </si>
-  <si>
-    <t>Delivery Success XPT</t>
-  </si>
-  <si>
-    <t>95.22%</t>
-  </si>
-  <si>
-    <t>94.75%</t>
-  </si>
-  <si>
-    <t>95.01%</t>
-  </si>
-  <si>
-    <t>94.54%</t>
-  </si>
-  <si>
-    <t>94.15%</t>
-  </si>
-  <si>
-    <t>89.00%</t>
-  </si>
-  <si>
-    <t>94.73%</t>
-  </si>
-  <si>
-    <t>% Real x D7 FDS (XPT) SPOT</t>
-  </si>
-  <si>
-    <t>100.00%</t>
-  </si>
-  <si>
-    <t>40.00%</t>
-  </si>
-  <si>
-    <t>80.00%</t>
-  </si>
-  <si>
-    <t>52.00%</t>
-  </si>
-  <si>
-    <t>Telemetria MM XPT</t>
-  </si>
-  <si>
-    <t>72.0%</t>
-  </si>
-  <si>
-    <t>54.00%</t>
-  </si>
-  <si>
-    <t>58.38%</t>
-  </si>
-  <si>
-    <t>63.55%</t>
-  </si>
-  <si>
-    <t>68.38%</t>
-  </si>
-  <si>
-    <t>67.91%</t>
-  </si>
-  <si>
-    <t>62.44%</t>
-  </si>
-  <si>
-    <t>Safety</t>
-  </si>
-  <si>
-    <t>Ad. Vec Fleet</t>
-  </si>
-  <si>
-    <t>84.00%</t>
-  </si>
-  <si>
-    <t>Telemetria Scorecard</t>
-  </si>
-  <si>
-    <t>88.17%</t>
-  </si>
-  <si>
-    <t>81.32%</t>
-  </si>
-  <si>
-    <t>87.47%</t>
-  </si>
-  <si>
-    <t>85.65%</t>
+    <t>102.10%</t>
   </si>
   <si>
     <t>Aderência Treinamentos Safety Driver</t>
   </si>
   <si>
-    <t>96.31%</t>
-  </si>
-  <si>
-    <t>95.17%</t>
-  </si>
-  <si>
-    <t>96.23%</t>
-  </si>
-  <si>
-    <t>96.83%</t>
-  </si>
-  <si>
-    <t>96.20%</t>
+    <t>95.87%</t>
+  </si>
+  <si>
+    <t>96.94%</t>
   </si>
   <si>
     <t>96.68%</t>
   </si>
   <si>
-    <t>96.15%</t>
+    <t>96.80%</t>
+  </si>
+  <si>
+    <t>96.41%</t>
+  </si>
+  <si>
+    <t>96.48%</t>
+  </si>
+  <si>
+    <t>96.54%</t>
   </si>
   <si>
     <t>Acompanhamento de Ações / Status das Tarefas</t>
@@ -420,25 +447,25 @@
     <t>Atrasado</t>
   </si>
   <si>
-    <t>Fechamento Semanal - BSC (W28)</t>
+    <t>Fechamento Semanal - BSC (Jun)</t>
   </si>
   <si>
     <t>Milha</t>
   </si>
   <si>
-    <t>W28 (Fechamento)</t>
+    <t>Jun (Fechamento)</t>
+  </si>
+  <si>
+    <t>Jul (Prévia)</t>
   </si>
   <si>
     <t>Aderência ao Perfil FULL</t>
   </si>
   <si>
-    <t>95.73%</t>
-  </si>
-  <si>
-    <t>93.13%</t>
-  </si>
-  <si>
-    <t>94.23%</t>
+    <t>Atingido</t>
+  </si>
+  <si>
+    <t>93.25%</t>
   </si>
   <si>
     <t>Aceite Scheduling Pré Routing</t>
@@ -447,20 +474,20 @@
     <t>5.0%</t>
   </si>
   <si>
-    <t>3.57%</t>
-  </si>
-  <si>
-    <t>4.39%</t>
-  </si>
-  <si>
-    <t>2.81%</t>
+    <t>4.60%</t>
+  </si>
+  <si>
+    <t>3.99%</t>
+  </si>
+  <si>
+    <t>3.46%</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -494,11 +521,11 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF00B050"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF00B050"/>
+      <color rgb="FFFF0000"/>
     </font>
     <font>
       <b/>
@@ -508,10 +535,6 @@
     <font>
       <b/>
       <color rgb="FF553C9A"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF000000"/>
     </font>
     <font>
       <b/>
@@ -588,7 +611,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -623,25 +646,22 @@
     <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1231,55 +1251,55 @@
         <v>15</v>
       </c>
       <c r="D6" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="F6" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="G6" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="H6" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="I6" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="J6" s="8" t="s">
+      <c r="J6" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="L6" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="L6" s="6" t="s">
+      <c r="M6" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="M6" s="7" t="s">
+      <c r="N6" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="N6" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="O6" s="8" t="s">
+      <c r="O6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="P6" s="8" t="s">
+      <c r="P6" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="Q6" s="8" t="s">
+      <c r="Q6" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="R6" s="8" t="s">
+      <c r="R6" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="S6" s="8" t="s">
+      <c r="S6" s="9" t="s">
         <v>29</v>
       </c>
       <c r="T6" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="U6" s="8" t="s">
-        <v>22</v>
+      <c r="U6" s="9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
@@ -1292,10 +1312,10 @@
       <c r="C7" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="8" t="s">
         <v>35</v>
       </c>
       <c r="F7" s="9" t="s">
@@ -1304,182 +1324,182 @@
       <c r="G7" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="H7" s="9" t="s">
         <v>38</v>
       </c>
       <c r="I7" s="7" t="s">
         <v>39</v>
       </c>
       <c r="J7" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="L7" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="L7" s="6" t="s">
+      <c r="M7" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="M7" s="7" t="s">
+      <c r="N7" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="N7" s="8" t="s">
+      <c r="O7" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="O7" s="8" t="s">
+      <c r="P7" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="P7" s="8" t="s">
+      <c r="Q7" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="Q7" s="8" t="s">
+      <c r="R7" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="S7" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="R7" s="8" t="s">
+      <c r="T7" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="S7" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="T7" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="U7" s="8" t="s">
-        <v>22</v>
+      <c r="U7" s="9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="D8" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="E8" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="F8" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="G8" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="H8" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="G8" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="H8" s="7" t="s">
+      <c r="I8" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="I8" s="7" t="s">
+      <c r="J8" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="L8" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="J8" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="L8" s="6" t="s">
+      <c r="M8" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="N8" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="M8" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="N8" s="9" t="s">
+      <c r="O8" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="O8" s="8" t="s">
+      <c r="P8" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="P8" s="8" t="s">
+      <c r="Q8" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="Q8" s="8" t="s">
+      <c r="R8" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="R8" s="8" t="s">
+      <c r="S8" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="S8" s="8" t="s">
+      <c r="T8" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="T8" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="U8" s="8" t="s">
-        <v>22</v>
+      <c r="U8" s="9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="D9" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="H9" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="J9" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="M9" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="N9" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="O9" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="H9" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="I9" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="L9" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="M9" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="N9" s="8" t="s">
+      <c r="P9" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="O9" s="8" t="s">
+      <c r="Q9" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="P9" s="8" t="s">
+      <c r="R9" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="Q9" s="8" t="s">
+      <c r="S9" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="R9" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="S9" s="8" t="s">
-        <v>75</v>
-      </c>
       <c r="T9" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="U9" s="8" t="s">
-        <v>22</v>
+        <v>56</v>
+      </c>
+      <c r="U9" s="9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C10" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="D10" s="8" t="s">
         <v>77</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>56</v>
       </c>
       <c r="E10" s="8" t="s">
         <v>78</v>
@@ -1490,76 +1510,76 @@
       <c r="G10" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="H10" s="8" t="s">
+      <c r="H10" s="9" t="s">
         <v>81</v>
       </c>
       <c r="I10" s="7" t="s">
         <v>82</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="L10" s="6" t="s">
         <v>83</v>
       </c>
       <c r="M10" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="N10" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="N10" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="O10" s="8" t="s">
+      <c r="O10" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="P10" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="P10" s="8" t="s">
+      <c r="Q10" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="Q10" s="8" t="s">
+      <c r="R10" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="R10" s="8" t="s">
+      <c r="S10" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="S10" s="8" t="s">
+      <c r="T10" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="T10" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="U10" s="8" t="s">
-        <v>22</v>
+      <c r="U10" s="9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="12:21" x14ac:dyDescent="0.25">
       <c r="L11" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="M11" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="N11" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="M11" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="N11" s="9" t="s">
+      <c r="O11" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="P11" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="O11" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="P11" s="8" t="s">
+      <c r="Q11" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="Q11" s="8" t="s">
+      <c r="R11" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="S11" s="9" t="s">
         <v>94</v>
-      </c>
-      <c r="R11" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="S11" s="8" t="s">
-        <v>48</v>
       </c>
       <c r="T11" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="U11" s="8" t="s">
-        <v>22</v>
+      <c r="U11" s="9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="12:21" x14ac:dyDescent="0.25">
@@ -1569,34 +1589,34 @@
       <c r="M12" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="N12" s="8" t="s">
+      <c r="N12" s="9" t="s">
         <v>98</v>
       </c>
       <c r="O12" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="P12" s="8" t="s">
+      <c r="P12" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="Q12" s="8" t="s">
+      <c r="Q12" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="R12" s="8" t="s">
+      <c r="R12" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="S12" s="7" t="s">
-        <v>56</v>
+      <c r="S12" s="9" t="s">
+        <v>103</v>
       </c>
       <c r="T12" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="U12" s="8" t="s">
-        <v>22</v>
+        <v>104</v>
+      </c>
+      <c r="U12" s="9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -1642,137 +1662,137 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="F15" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>56</v>
+        <v>41</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>110</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>56</v>
+        <v>111</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="J15" s="12" t="s">
-        <v>56</v>
+        <v>112</v>
+      </c>
+      <c r="J15" s="9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>56</v>
+        <v>114</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>115</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="G16" s="7" t="s">
-        <v>56</v>
+        <v>117</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>119</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>56</v>
+        <v>111</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="J16" s="12" t="s">
-        <v>56</v>
+        <v>120</v>
+      </c>
+      <c r="J16" s="9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="G17" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="H17" s="8" t="s">
-        <v>118</v>
+        <v>75</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="H17" s="9" t="s">
+        <v>127</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="J17" s="8" t="s">
-        <v>22</v>
+        <v>128</v>
+      </c>
+      <c r="J17" s="9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="13"/>
-      <c r="H21" s="13"/>
-      <c r="I21" s="13"/>
-      <c r="J21" s="13"/>
-      <c r="K21" s="13"/>
+      <c r="A21" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="12"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="14" t="s">
-        <v>121</v>
-      </c>
-      <c r="B22" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14" t="s">
-        <v>124</v>
-      </c>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="I22" s="14"/>
-      <c r="J22" s="14"/>
-      <c r="K22" s="14" t="s">
+      <c r="A22" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="G22" s="13"/>
+      <c r="H22" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="I22" s="13"/>
+      <c r="J22" s="13"/>
+      <c r="K22" s="13" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1781,24 +1801,24 @@
         <v>2</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
       <c r="F23" s="7" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="G23" s="7"/>
       <c r="H23" s="7" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="I23" s="7"/>
       <c r="J23" s="7"/>
       <c r="K23" s="7" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -1809,46 +1829,46 @@
         <v>96</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="D24" s="6"/>
       <c r="E24" s="6"/>
       <c r="F24" s="7" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="G24" s="7"/>
       <c r="H24" s="7" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="I24" s="7"/>
       <c r="J24" s="7"/>
       <c r="K24" s="7" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="D25" s="6"/>
       <c r="E25" s="6"/>
       <c r="F25" s="7" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="G25" s="7"/>
       <c r="H25" s="7" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="I25" s="7"/>
       <c r="J25" s="7"/>
-      <c r="K25" s="8" t="s">
-        <v>134</v>
+      <c r="K25" s="9" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -1890,89 +1910,89 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
-        <v>135</v>
-      </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
+      <c r="A1" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="15"/>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
     </row>
     <row r="4" ht="25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
-        <v>136</v>
-      </c>
-      <c r="B4" s="16" t="s">
+      <c r="A4" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="B4" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="16" t="s">
-        <v>137</v>
-      </c>
-      <c r="F4" s="16" t="s">
+      <c r="E4" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="F4" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="16" t="s">
-        <v>10</v>
+      <c r="G4" s="15" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="8" t="s">
+      <c r="D5" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" s="7" t="s">
         <v>19</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="17" t="s">
         <v>39</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>37</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>38</v>
@@ -1982,89 +2002,89 @@
       <c r="A7" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="D7" s="18" t="s">
-        <v>139</v>
+      <c r="B7" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" s="17" t="s">
+        <v>69</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>140</v>
+        <v>18</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>22</v>
+        <v>149</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="D8" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>22</v>
+      <c r="B8" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>73</v>
-      </c>
-      <c r="E9" s="8" t="s">
+      <c r="B9" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G9" s="7" t="s">
         <v>71</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="17" t="s">
-        <v>76</v>
-      </c>
-      <c r="C10" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="D10" s="18" t="s">
+      <c r="B10" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" s="17" t="s">
         <v>82</v>
       </c>
       <c r="E10" s="9" t="s">
         <v>80</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="G10" s="7" t="s">
         <v>81</v>
@@ -2074,20 +2094,20 @@
       <c r="A11" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="D11" s="18" t="s">
+      <c r="D11" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="8" t="s">
-        <v>22</v>
+      <c r="F11" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="G11" s="7" t="s">
         <v>29</v>
@@ -2097,230 +2117,230 @@
       <c r="A12" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="E12" s="8" t="s">
+      <c r="D12" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="F12" s="8" t="s">
-        <v>22</v>
+      <c r="E12" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B13" s="17" t="s">
-        <v>142</v>
-      </c>
-      <c r="C13" s="18" t="s">
-        <v>143</v>
-      </c>
-      <c r="D13" s="18" t="s">
-        <v>144</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>22</v>
+      <c r="B13" s="16" t="s">
+        <v>151</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>152</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>153</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B14" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="C14" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="E14" s="8" t="s">
+      <c r="B14" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G14" s="7" t="s">
         <v>63</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B15" s="17" t="s">
-        <v>74</v>
-      </c>
-      <c r="C15" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="D15" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="F15" s="8" t="s">
-        <v>22</v>
+      <c r="B15" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>75</v>
+        <v>55</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="C16" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="D16" s="18" t="s">
-        <v>90</v>
-      </c>
-      <c r="E16" s="8" t="s">
+      <c r="C16" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="D16" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G16" s="7" t="s">
         <v>88</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="G16" s="7" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B17" s="17" t="s">
-        <v>91</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="D17" s="18" t="s">
+      <c r="B17" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="C17" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D17" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="F17" s="8" t="s">
-        <v>22</v>
+      <c r="F17" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>48</v>
+        <v>94</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="C18" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="D18" s="18" t="s">
+      <c r="D18" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" s="7" t="s">
         <v>103</v>
-      </c>
-      <c r="E18" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="G18" s="7" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="B19" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="C19" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="D19" s="18" t="s">
+      <c r="B19" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="E19" s="18" t="s">
-        <v>56</v>
-      </c>
-      <c r="F19" s="12" t="s">
-        <v>56</v>
+      <c r="C19" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D19" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>56</v>
+        <v>111</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="B20" s="17" t="s">
-        <v>107</v>
-      </c>
-      <c r="C20" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="D20" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="D20" s="17" t="s">
+        <v>120</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G20" s="7" t="s">
         <v>111</v>
-      </c>
-      <c r="E20" s="18" t="s">
-        <v>56</v>
-      </c>
-      <c r="F20" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="G20" s="7" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="B21" s="17" t="s">
-        <v>112</v>
-      </c>
-      <c r="C21" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="D21" s="18" t="s">
-        <v>119</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="F21" s="8" t="s">
-        <v>22</v>
+        <v>105</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="C21" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>